<commit_message>
Nesta aula fizemos a atividade"Banco tabajara"
</commit_message>
<xml_diff>
--- a/BANCO/cadastro_clinetes.xlsx
+++ b/BANCO/cadastro_clinetes.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,31 +432,278 @@
           <t>conta_cliente</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>numero_conta</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>agencia</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>extrato</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Israel</t>
+          <t>Israel vinicius</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>444</v>
-      </c>
-      <c r="C2" t="n">
-        <v>2</v>
+        <v>5555</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Corrente</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" t="n">
+        <v>400</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>israel</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>555</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Poupança</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" t="n">
+        <v>400</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>israel</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>4444</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Salário</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" t="n">
+        <v>400</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>israel Moura</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>5555</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Salário</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" t="n">
+        <v>400</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
           <t>Israel</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="B6" t="n">
         <v>5555</v>
       </c>
-      <c r="C3" t="n">
-        <v>3</v>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Salário</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Israel</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>5555</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Salário</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>israel</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>5555</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Corrente</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>7</v>
+      </c>
+      <c r="E8" t="n">
+        <v>406</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Israel</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>5555</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Poupança</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>8</v>
+      </c>
+      <c r="E9" t="n">
+        <v>407</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Israel feliz</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>5555</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Poupança</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>9</v>
+      </c>
+      <c r="E10" t="n">
+        <v>408</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Israel</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>5555</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Salário</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>10</v>
+      </c>
+      <c r="E11" t="n">
+        <v>409</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Israel</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>55555</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Corrente</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>11</v>
+      </c>
+      <c r="E12" t="n">
+        <v>410</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Nesta aula foi passado a segunda perto do exercicio!
</commit_message>
<xml_diff>
--- a/BANCO/cadastro_clinetes.xlsx
+++ b/BANCO/cadastro_clinetes.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -451,11 +451,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Israel vinicius</t>
+          <t>Israel Albuquerque</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>5555</v>
+        <v>555</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -463,247 +463,61 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E2" t="n">
         <v>400</v>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>199979</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>israel</t>
+          <t>Maria Jose</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>555</v>
+        <v>222</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Poupança</t>
+          <t>Salário</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E3" t="n">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>300000</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>israel</t>
+          <t>Jose Almeida</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>4444</v>
+        <v>888</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Salário</t>
+          <t>Poupança</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E4" t="n">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="F4" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>israel Moura</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>5555</v>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Salário</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E5" t="n">
-        <v>400</v>
-      </c>
-      <c r="F5" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Israel</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>5555</v>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Salário</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F6" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Israel</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>5555</v>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Salário</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>israel</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>5555</v>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Corrente</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
-        <v>7</v>
-      </c>
-      <c r="E8" t="n">
-        <v>406</v>
-      </c>
-      <c r="F8" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Israel</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>5555</v>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Poupança</t>
-        </is>
-      </c>
-      <c r="D9" t="n">
-        <v>8</v>
-      </c>
-      <c r="E9" t="n">
-        <v>407</v>
-      </c>
-      <c r="F9" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Israel feliz</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>5555</v>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Poupança</t>
-        </is>
-      </c>
-      <c r="D10" t="n">
-        <v>9</v>
-      </c>
-      <c r="E10" t="n">
-        <v>408</v>
-      </c>
-      <c r="F10" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Israel</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>5555</v>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Salário</t>
-        </is>
-      </c>
-      <c r="D11" t="n">
-        <v>10</v>
-      </c>
-      <c r="E11" t="n">
-        <v>409</v>
-      </c>
-      <c r="F11" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Israel</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>55555</v>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Corrente</t>
-        </is>
-      </c>
-      <c r="D12" t="n">
-        <v>11</v>
-      </c>
-      <c r="E12" t="n">
-        <v>410</v>
-      </c>
-      <c r="F12" t="n">
-        <v>0</v>
+        <v>500000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Nesta aula ouve o termino da atividade do banco tabajara.
</commit_message>
<xml_diff>
--- a/BANCO/cadastro_clinetes.xlsx
+++ b/BANCO/cadastro_clinetes.xlsx
@@ -469,7 +469,7 @@
         <v>400</v>
       </c>
       <c r="F2" t="n">
-        <v>199979</v>
+        <v>300855</v>
       </c>
     </row>
     <row r="3">
@@ -493,7 +493,7 @@
         <v>401</v>
       </c>
       <c r="F3" t="n">
-        <v>300000</v>
+        <v>299898</v>
       </c>
     </row>
     <row r="4">
@@ -517,7 +517,7 @@
         <v>402</v>
       </c>
       <c r="F4" t="n">
-        <v>500000</v>
+        <v>500100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>